<commit_message>
feat(jurisdictions/sg): FRTB SA(MR), DRC, RRAO, IMA scalars and SSA(MR) (MAS Notice 637 Part VIII)
The comparison now runs all six regimes on their own FRTB engines; only
capital resources are held common.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BMvrGqjRYkJu5447z7YL4q
</commit_message>
<xml_diff>
--- a/output/reports/e2e/E2E_Results.xlsx
+++ b/output/reports/e2e/E2E_Results.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.016</v>
+        <v>0.01</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.019</v>
+        <v>0.013</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.17</v>
+        <v>0.168</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.606</v>
+        <v>0.611</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.466</v>
+        <v>0.654</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1794,18 +1794,22 @@
         <v>331502.8314298259</v>
       </c>
       <c r="M6" t="n">
-        <v>204466.0667840441</v>
+        <v>206232.795394049</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>16414.44813474237</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>4.175496781551914</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
       <c r="R6" t="n">
         <v>48500</v>
       </c>
@@ -1816,7 +1820,7 @@
         <v>7377.5</v>
       </c>
       <c r="U6" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="b">
@@ -1829,16 +1833,16 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925435</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.1172243055227626</v>
+        <v>0.1171077025463321</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.1307501869292352</v>
+        <v>0.1306201297632165</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.1570267228713577</v>
+        <v>0.1568705284440649</v>
       </c>
       <c r="AD6" t="n">
         <v>3753092.761918609</v>
@@ -1859,7 +1863,7 @@
         <v>0.11</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.00722430552276257</v>
+        <v>0.007107702546332056</v>
       </c>
       <c r="AK6" t="n">
         <v>0.03</v>
@@ -2705,18 +2709,22 @@
         <v>331502.8314298259</v>
       </c>
       <c r="M6" t="n">
-        <v>204466.0667840441</v>
+        <v>206232.795394049</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>16414.44813474237</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>4.175496781551914</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
       <c r="R6" t="n">
         <v>48500</v>
       </c>
@@ -2727,7 +2735,7 @@
         <v>7377.5</v>
       </c>
       <c r="U6" t="n">
-        <v>1780190.084801815</v>
+        <v>1781956.81341182</v>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="b">
@@ -2740,16 +2748,16 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>1780190.084801815</v>
+        <v>1781956.81341182</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.1168414551770499</v>
+        <v>0.1167256122227526</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.1303231615436326</v>
+        <v>0.1301939520946086</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.1565138792689211</v>
+        <v>0.1563587029221735</v>
       </c>
       <c r="AD6" t="n">
         <v>3753092.761918609</v>
@@ -2770,7 +2778,7 @@
         <v>0.11</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.006841455177049913</v>
+        <v>0.006725612222752558</v>
       </c>
       <c r="AK6" t="n">
         <v>0.03</v>
@@ -6673,7 +6681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6996,7 +7004,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7005,13 +7013,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4427.009268437907</v>
+        <v>4427.009268437909</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7020,13 +7028,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9787.49380555365</v>
+        <v>9787.493805553651</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7041,7 +7049,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7056,15 +7064,90 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FX</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>237.2787670821237</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>GIRR</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>4427.009268437907</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CSR_NONSEC</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>9787.49380555365</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>902.8587176988991</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1059.807575969784</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>FX</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C31" t="n">
         <v>237.2787670821237</v>
       </c>
     </row>
@@ -7585,16 +7668,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G14" t="n">
-        <v>887188.0241577147</v>
+        <v>888071.3884627172</v>
       </c>
       <c r="H14" t="n">
-        <v>1153344.431405029</v>
+        <v>1154492.805001533</v>
       </c>
       <c r="I14" t="n">
-        <v>266156.4072473145</v>
+        <v>266421.4165388153</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -7621,16 +7704,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G15" t="n">
-        <v>1064625.628989258</v>
+        <v>1065685.666155261</v>
       </c>
       <c r="H15" t="n">
-        <v>1153344.431405029</v>
+        <v>1154492.805001533</v>
       </c>
       <c r="I15" t="n">
-        <v>88718.80241577154</v>
+        <v>88807.13884627205</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -7657,13 +7740,13 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G16" t="n">
-        <v>1242063.2338208</v>
+        <v>1243299.943847804</v>
       </c>
       <c r="H16" t="n">
-        <v>1242063.2338208</v>
+        <v>1243299.943847804</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -8233,16 +8316,16 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G32" t="n">
-        <v>887188.0241577147</v>
+        <v>888071.3884627172</v>
       </c>
       <c r="H32" t="n">
-        <v>1286422.635028686</v>
+        <v>1287703.51327094</v>
       </c>
       <c r="I32" t="n">
-        <v>399234.6108709715</v>
+        <v>399632.1248082228</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -8269,16 +8352,16 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G33" t="n">
-        <v>1064625.628989258</v>
+        <v>1065685.666155261</v>
       </c>
       <c r="H33" t="n">
-        <v>1286422.635028686</v>
+        <v>1287703.51327094</v>
       </c>
       <c r="I33" t="n">
-        <v>221797.0060394286</v>
+        <v>222017.8471156795</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -8305,16 +8388,16 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1774376.048315429</v>
+        <v>1776142.776925434</v>
       </c>
       <c r="G34" t="n">
-        <v>1242063.2338208</v>
+        <v>1243299.943847804</v>
       </c>
       <c r="H34" t="n">
-        <v>1286422.635028686</v>
+        <v>1287703.51327094</v>
       </c>
       <c r="I34" t="n">
-        <v>44359.40120788569</v>
+        <v>44403.56942313611</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>

</xml_diff>